<commit_message>
Polish practicals across the site and add the Sklad+ kit
- reorder MDK.03.02 so lectures come before practices
- add specialty names for 09.02.12 and 09.02.13
- rename MDK.06.01 and MDK.06.02 practices to adjacent topics
- remove third-person student wording from lesson descriptions
- switch practical criteria to a 1-5 scale with the AI and copy rule
- replace absolute file paths with relative paths
- add a starter kit for MDK.06.01: prototype, SQL, data and templates
- rewrite practical tables so students work from raw data, not ready answers
</commit_message>
<xml_diff>
--- a/courses/3/is-code/dist/Учебный_план_Разработка_кода_информационных_систем.xlsx
+++ b/courses/3/is-code/dist/Учебный_план_Разработка_кода_информационных_систем.xlsx
@@ -195,7 +195,7 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Место разработки кода в жизненном цикле информационной системы: от требований до сопровождения. Студент разберёт роли в команде и получит карту всего курса.</t>
+          <t xml:space="preserve">Место разработки кода в жизненном цикле информационной системы: от требований до сопровождения. Вы разберёте роли в команде и получите карту всего курса.</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
@@ -204,7 +204,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="60" customHeight="1">
+    <row r="7" ht="45" customHeight="1">
       <c r="A7" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">2</t>
@@ -225,7 +225,7 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Три слоя приложения: интерфейс, бизнес-логика и доступ к данным. Студент научится раскладывать функции системы по слоям и объяснять связи между ними.</t>
+          <t xml:space="preserve">Три слоя приложения: интерфейс, бизнес-логика и доступ к данным. Вы научитесь раскладывать функции системы по слоям и объяснять связи между ними.</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
@@ -255,7 +255,7 @@
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Каталоги src, tests и docs, файлы конфигурации и список зависимостей. Студент соберёт каркас проекта, в котором код, тесты и данные лежат на своих местах.</t>
+          <t xml:space="preserve">Каталоги src, tests и docs, файлы конфигурации и список зависимостей. Вы соберёте каркас проекта, в котором код, тесты и данные лежат на своих местах.</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
@@ -285,7 +285,7 @@
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Запуск Python-файла, виртуальное окружение, терминал и отладчик в VS Code. Студент выполнит первую программу и настроит окружение без глобальных установок.</t>
+          <t xml:space="preserve">Запуск Python-файла, виртуальное окружение, терминал и отладчик в VS Code. Вы выполните первую программу и настроите окружение без глобальных установок.</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">
@@ -315,7 +315,7 @@
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Студент создаёт каркас проекта, пишет модуль расчёта на Python с вводом и выводом, раскладывает функции по файлам и сдаёт репозиторий с README.</t>
+          <t xml:space="preserve">Вы создаёте каркас проекта, пишете модуль расчёта на Python с вводом и выводом, раскладываете функции по файлам и сдаёте репозиторий с README.</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
@@ -345,7 +345,7 @@
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Устройство решения и проекта C#, сборка через .NET CLI и запуск консольного приложения. Студент сравнит цикл правки и запуска в C# и Python.</t>
+          <t xml:space="preserve">Устройство решения и проекта C#, сборка через .NET CLI и запуск консольного приложения. Вы сравните цикл правки и запуска в C# и Python.</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr">
@@ -375,7 +375,7 @@
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Студент ставит расширения Python и C#, настраивает интерпретатор, форматирование и отладчик в двух редакторах, сдаёт скриншоты настроек и запущенный проект.</t>
+          <t xml:space="preserve">Вы ставите расширения Python и C#, настраиваете интерпретатор, форматирование и отладчик в двух редакторах, сдаёте скриншоты настроек и запущенный проект.</t>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr">
@@ -384,7 +384,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="60" customHeight="1">
+    <row r="13" ht="45" customHeight="1">
       <c r="A13" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">10</t>
@@ -405,7 +405,7 @@
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Типы данных, объявление переменных и преобразование значений в Python и C#. Студент разберёт, откуда берутся ошибки приведения типов и как их избежать.</t>
+          <t xml:space="preserve">Типы данных, объявление переменных и преобразование значений в Python и C#. Вы разберёте, откуда берутся ошибки приведения типов и как их избежать.</t>
         </is>
       </c>
       <c r="F13" s="5" t="inlineStr">
@@ -435,7 +435,7 @@
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ветвления, циклы и обработка коллекций в двух языках. Студент научится выбирать конструкцию под задачу и переводить алгоритм с Python на C#.</t>
+          <t xml:space="preserve">Ветвления, циклы и обработка коллекций в двух языках. Вы научитесь выбирать конструкцию под задачу и переводить алгоритм с Python на C#.</t>
         </is>
       </c>
       <c r="F14" s="5" t="inlineStr">
@@ -465,7 +465,7 @@
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Параметры, возврат значения, области видимости и вынос кода в модуль. Студент разберёт, как отдельная функция превращается в переиспользуемый модуль проекта.</t>
+          <t xml:space="preserve">Параметры, возврат значения, области видимости и вынос кода в модуль. Вы разберёте, как отдельная функция превращается в переиспользуемый модуль проекта.</t>
         </is>
       </c>
       <c r="F15" s="5" t="inlineStr">
@@ -495,7 +495,7 @@
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Студент пишет консольную программу на C# с методами, параметрами и возвратом значения, разбивает её на файлы и сдаёт проект, который собирается без предупреждений.</t>
+          <t xml:space="preserve">Вы пишете консольную программу на C# с методами, параметрами и возвратом значения, разбиваете её на файлы и сдаёте проект, который собирается без предупреждений.</t>
         </is>
       </c>
       <c r="F16" s="5" t="inlineStr">
@@ -525,7 +525,7 @@
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Наследование, инкапсуляция и полиморфизм на примере иерархии сущностей. Студент увидит, когда классы стоит объединять общим родителем, а когда нет.</t>
+          <t xml:space="preserve">Наследование, инкапсуляция и полиморфизм на примере иерархии сущностей. Вы увидите, когда классы стоит объединять общим родителем, а когда нет.</t>
         </is>
       </c>
       <c r="F17" s="5" t="inlineStr">
@@ -534,7 +534,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="60" customHeight="1">
+    <row r="18" ht="45" customHeight="1">
       <c r="A18" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">16</t>
@@ -555,7 +555,7 @@
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Студент описывает класс предметной области с полями, конструктором и методами, создаёт несколько объектов и сдаёт программу с проверкой их состояния.</t>
+          <t xml:space="preserve">Вы описываете класс предметной области с полями, конструктором и методами, создаёте несколько объектов и сдаёте программу с проверкой их состояния.</t>
         </is>
       </c>
       <c r="F18" s="5" t="inlineStr">
@@ -564,7 +564,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="60" customHeight="1">
+    <row r="19" ht="45" customHeight="1">
       <c r="A19" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">17</t>
@@ -585,7 +585,7 @@
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Иерархия исключений, собственные классы ошибок и стратегия обработки на границах модуля. Студент научится не глотать ошибку и сохранять причину сбоя.</t>
+          <t xml:space="preserve">Иерархия исключений, собственные классы ошибок и стратегия обработки на границах модуля. Вы научитесь не глотать ошибку и сохранять причину сбоя.</t>
         </is>
       </c>
       <c r="F19" s="5" t="inlineStr">
@@ -615,7 +615,7 @@
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Студент добавляет в программу обработку ошибочных ситуаций: проверяет ввод, перехватывает исключения и сдаёт код, который не падает на пустом или неверном значении.</t>
+          <t xml:space="preserve">Вы добавляете в программу обработку ошибочных ситуаций: проверяете ввод, перехватываете исключения и сдаёте код, который не падает на пустом или неверном значении.</t>
         </is>
       </c>
       <c r="F20" s="5" t="inlineStr">
@@ -645,7 +645,7 @@
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Пути, кодировки, построчное чтение больших файлов и контекстный менеджер. Студент разберёт, почему файл теряет данные и как этого не допустить.</t>
+          <t xml:space="preserve">Пути, кодировки, построчное чтение больших файлов и контекстный менеджер. Вы разберёте, почему файл теряет данные и как этого не допустить.</t>
         </is>
       </c>
       <c r="F21" s="5" t="inlineStr">
@@ -675,7 +675,7 @@
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Студент читает и записывает текстовый файл, добавляет строки и обрабатывает отсутствие файла, сдаёт программу с журналом операций в файле.</t>
+          <t xml:space="preserve">Вы читаете и записываете текстовый файл, добавляете строки и обрабатываете отсутствие файла, сдаёте программу с журналом операций в файле.</t>
         </is>
       </c>
       <c r="F22" s="5" t="inlineStr">
@@ -684,7 +684,7 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="60" customHeight="1">
+    <row r="23" ht="45" customHeight="1">
       <c r="A23" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">21</t>
@@ -705,7 +705,7 @@
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Форматы обмена данными: вложенность JSON, заголовок CSV, типы значений после разбора. Студент научится выбирать формат под задачу импорта и экспорта.</t>
+          <t xml:space="preserve">Форматы обмена данными: вложенность JSON, заголовок CSV, типы значений после разбора. Вы научитесь выбирать формат под задачу импорта и экспорта.</t>
         </is>
       </c>
       <c r="F23" s="5" t="inlineStr">
@@ -735,7 +735,7 @@
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Студент читает JSON и CSV, преобразует записи в объекты программы, фильтрует их и сохраняет результат в новый файл, сдаёт скрипт и оба файла данных.</t>
+          <t xml:space="preserve">Вы читаете JSON и CSV, преобразуете записи в объекты программы, фильтруете их и сохраняете результат в новый файл, сдаёте скрипт и оба файла данных.</t>
         </is>
       </c>
       <c r="F24" s="5" t="inlineStr">
@@ -744,7 +744,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="60" customHeight="1">
+    <row r="25" ht="45" customHeight="1">
       <c r="A25" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">23</t>
@@ -765,7 +765,7 @@
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Устройство файловой базы SQLite: таблицы, индексы, транзакции и ограничения целостности. Студент прочитает схему учебной базы и объяснит связи в ней.</t>
+          <t xml:space="preserve">Устройство файловой базы SQLite: таблицы, индексы, транзакции и ограничения целостности. Вы прочитаете схему учебной базы и объясните связи в ней.</t>
         </is>
       </c>
       <c r="F25" s="5" t="inlineStr">
@@ -795,7 +795,7 @@
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Студент создаёт базу SQLite, таблицы с первичным и внешним ключом, заполняет их и сдаёт файл базы вместе со скриптом создания схемы.</t>
+          <t xml:space="preserve">Вы создаёте базу SQLite, таблицы с первичным и внешним ключом, заполняете их и сдаёте файл базы вместе со скриптом создания схемы.</t>
         </is>
       </c>
       <c r="F26" s="5" t="inlineStr">
@@ -804,7 +804,7 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="60" customHeight="1">
+    <row r="27" ht="45" customHeight="1">
       <c r="A27" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">25</t>
@@ -825,7 +825,7 @@
       </c>
       <c r="E27" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Параметризованные запросы, чтение строк в объекты и обработка пустого результата. Студент разберёт разницу между склейкой строки и параметром запроса.</t>
+          <t xml:space="preserve">Параметризованные запросы, чтение строк в объекты и обработка пустого результата. Вы разберёте разницу между склейкой строки и параметром запроса.</t>
         </is>
       </c>
       <c r="F27" s="5" t="inlineStr">
@@ -855,7 +855,7 @@
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Студент подключает базу SQLite из Python, выполняет SELECT, INSERT и UPDATE с параметрами и сдаёт скрипт, который наполняет базу и выводит отчёт.</t>
+          <t xml:space="preserve">Вы подключаете базу SQLite из Python, выполняете SELECT, INSERT и UPDATE с параметрами и сдаёте скрипт, который наполняет базу и выводит отчёт.</t>
         </is>
       </c>
       <c r="F28" s="5" t="inlineStr">
@@ -885,7 +885,7 @@
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Модель таблицы как класс, сессия и запросы вместо ручного SQL. Студент сравнит ORM и чистый SQL и увидит, где какой подход уместен.</t>
+          <t xml:space="preserve">Модель таблицы как класс, сессия и запросы вместо ручного SQL. Вы сравните ORM и чистый SQL и увидите, где какой подход уместен.</t>
         </is>
       </c>
       <c r="F29" s="5" t="inlineStr">
@@ -915,7 +915,7 @@
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Методы HTTP, заголовки, коды состояния и структура REST-ресурса. Студент проследит путь запроса от клиента до ответа и научится читать ответ API.</t>
+          <t xml:space="preserve">Методы HTTP, заголовки, коды состояния и структура REST-ресурса. Вы проследите путь запроса от клиента до ответа и научитесь читать ответ API.</t>
         </is>
       </c>
       <c r="F30" s="5" t="inlineStr">
@@ -945,7 +945,7 @@
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Сравнение двух Python-фреймворков: маршруты, схемы данных и автоматическая документация. Студент выберет фреймворк под задачу и обоснует выбор.</t>
+          <t xml:space="preserve">Сравнение двух Python-фреймворков: маршруты, схемы данных и автоматическая документация. Вы выберете фреймворк под задачу и обоснуете выбор.</t>
         </is>
       </c>
       <c r="F31" s="5" t="inlineStr">
@@ -975,7 +975,7 @@
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Студент запускает Flask-сервис с двумя маршрутами, обращается к нему из HTTP-клиента и Postman и сдаёт коллекцию запросов с ответами и кодами состояния.</t>
+          <t xml:space="preserve">Вы запускаете Flask-сервис с двумя маршрутами, обращаетесь к нему из HTTP-клиента и Postman и сдаёте коллекцию запросов с ответами и кодами состояния.</t>
         </is>
       </c>
       <c r="F32" s="5" t="inlineStr">
@@ -1005,7 +1005,7 @@
       </c>
       <c r="E33" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Устройство приложения ASP.NET Core: конвейер обработки запроса, внедрение зависимостей и конфигурация. Студент разберёт, где подключить сервис и middleware.</t>
+          <t xml:space="preserve">Устройство приложения ASP.NET Core: конвейер обработки запроса, внедрение зависимостей и конфигурация. Вы разберёте, где подключить сервис и middleware.</t>
         </is>
       </c>
       <c r="F33" s="5" t="inlineStr">
@@ -1035,7 +1035,7 @@
       </c>
       <c r="E34" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Студент создаёт контроллер ASP.NET с маршрутами чтения и записи, подключает хранилище и сдаёт работающий сервис с проверкой запросов в Postman.</t>
+          <t xml:space="preserve">Вы создаёте контроллер ASP.NET с маршрутами чтения и записи, подключаете хранилище и сдаёте работающий сервис с проверкой запросов в Postman.</t>
         </is>
       </c>
       <c r="F34" s="5" t="inlineStr">
@@ -1065,7 +1065,7 @@
       </c>
       <c r="E35" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Аутентификация и авторизация, хранение паролей и выдача токена. Студент разберёт поток входа и типичные ошибки при проверке прав доступа.</t>
+          <t xml:space="preserve">Аутентификация и авторизация, хранение паролей и выдача токена. Вы разберёте поток входа и типичные ошибки при проверке прав доступа.</t>
         </is>
       </c>
       <c r="F35" s="5" t="inlineStr">
@@ -1074,7 +1074,7 @@
         </is>
       </c>
     </row>
-    <row r="36" ht="60" customHeight="1">
+    <row r="36" ht="45" customHeight="1">
       <c r="A36" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">35</t>
@@ -1095,7 +1095,7 @@
       </c>
       <c r="E36" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Основные угрозы веб-приложения: инъекции, утечка секретов и слабая проверка доступа. Студент научится находить уязвимость в коде и предлагать защиту.</t>
+          <t xml:space="preserve">Основные угрозы веб-приложения: инъекции, утечка секретов и слабая проверка доступа. Вы научитесь находить уязвимость в коде и предлагать защиту.</t>
         </is>
       </c>
       <c r="F36" s="5" t="inlineStr">
@@ -1125,7 +1125,7 @@
       </c>
       <c r="E37" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Проверка данных на входе, в модели и в базе: обязательность, длина, диапазон и формат. Студент построит правило проверки и вернёт понятное сообщение об ошибке.</t>
+          <t xml:space="preserve">Проверка данных на входе, в модели и в базе: обязательность, длина, диапазон и формат. Вы построите правило проверки и вернёте понятное сообщение об ошибке.</t>
         </is>
       </c>
       <c r="F37" s="5" t="inlineStr">
@@ -1155,7 +1155,7 @@
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Студент добавляет в API вход по логину и паролю, проверку токена и валидацию полей, сдаёт сервис, который отклоняет неверные данные с понятным кодом ошибки.</t>
+          <t xml:space="preserve">Вы добавляете в API вход по логину и паролю, проверку токена и валидацию полей, сдаёте сервис, который отклоняет неверные данные с понятным кодом ошибки.</t>
         </is>
       </c>
       <c r="F38" s="5" t="inlineStr">
@@ -1185,7 +1185,7 @@
       </c>
       <c r="E39" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Уровни сообщений, формат записи и место хранения журнала. Студент настроит логирование так, чтобы по записи можно было восстановить ход запроса.</t>
+          <t xml:space="preserve">Уровни сообщений, формат записи и место хранения журнала. Вы настроите логирование так, чтобы по записи можно было восстановить ход запроса.</t>
         </is>
       </c>
       <c r="F39" s="5" t="inlineStr">
@@ -1215,7 +1215,7 @@
       </c>
       <c r="E40" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Студент закрывает уязвимые места сервиса: убирает секреты из кода, включает проверку ввода и пишет события в журнал, сдаёт отчёт о проверке и файл лога.</t>
+          <t xml:space="preserve">Вы закрываете уязвимые места сервиса: убираете секреты из кода, включаете проверку ввода и пишете события в журнал, сдаёте отчёт о проверке и файл лога.</t>
         </is>
       </c>
       <c r="F40" s="5" t="inlineStr">
@@ -1245,7 +1245,7 @@
       </c>
       <c r="E41" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Модульные и интеграционные тесты, покрытие и граничные значения. Студент научится отличать проверку одной функции от проверки связки модулей.</t>
+          <t xml:space="preserve">Модульные и интеграционные тесты, покрытие и граничные значения. Вы научитесь отличать проверку одной функции от проверки связки модулей.</t>
         </is>
       </c>
       <c r="F41" s="5" t="inlineStr">
@@ -1275,7 +1275,7 @@
       </c>
       <c r="E42" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Точки останова, пошаговое выполнение и просмотр стека вызовов в VS Code и Visual Studio. Студент найдёт причину дефекта без правок наугад.</t>
+          <t xml:space="preserve">Точки останова, пошаговое выполнение и просмотр стека вызовов в VS Code и Visual Studio. Вы найдёте причину дефекта без правок наугад.</t>
         </is>
       </c>
       <c r="F42" s="5" t="inlineStr">
@@ -1305,7 +1305,7 @@
       </c>
       <c r="E43" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Студент пишет тесты на функцию и на маршрут API, запускает их и находит дефект по падающему тесту, сдаёт набор тестов и короткий отчёт о причине сбоя.</t>
+          <t xml:space="preserve">Вы пишете тесты на функцию и на маршрут API, запускаете их и находите дефект по падающему тесту, сдаёте набор тестов и короткий отчёт о причине сбоя.</t>
         </is>
       </c>
       <c r="F43" s="5" t="inlineStr">
@@ -1335,7 +1335,7 @@
       </c>
       <c r="E44" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ветки, слияние и разрешение конфликтов в общем репозитории. Студент разберёт схему ветвления и научится сводить изменения без потери чужой работы.</t>
+          <t xml:space="preserve">Ветки, слияние и разрешение конфликтов в общем репозитории. Вы разберёте схему ветвления и научитесь сводить изменения без потери чужой работы.</t>
         </is>
       </c>
       <c r="F44" s="5" t="inlineStr">
@@ -1365,7 +1365,7 @@
       </c>
       <c r="E45" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Студент инициализирует репозиторий, делает серию коммитов, отправляет проект на GitHub и сдаёт ссылку на репозиторий с историей изменений.</t>
+          <t xml:space="preserve">Вы инициализируете репозиторий, делаете серию коммитов, отправляете проект на GitHub и сдаёте ссылку на репозиторий с историей изменений.</t>
         </is>
       </c>
       <c r="F45" s="5" t="inlineStr">
@@ -1374,7 +1374,7 @@
         </is>
       </c>
     </row>
-    <row r="46" ht="60" customHeight="1">
+    <row r="46" ht="45" customHeight="1">
       <c r="A46" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">48</t>
@@ -1395,7 +1395,7 @@
       </c>
       <c r="E46" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Цели рецензирования, чек-лист и культура замечаний. Студент разберёт, чем полезное замечание отличается от придирки, и потренируется на фрагменте кода.</t>
+          <t xml:space="preserve">Цели рецензирования, чек-лист и культура замечаний. Вы разберёте, чем полезное замечание отличается от придирки, и потренируетесь на фрагменте кода.</t>
         </is>
       </c>
       <c r="F46" s="5" t="inlineStr">
@@ -1425,7 +1425,7 @@
       </c>
       <c r="E47" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Менеджеры пакетов, файлы зависимостей и воспроизводимая сборка. Студент разберёт, почему проект работает на одной машине и падает на другой.</t>
+          <t xml:space="preserve">Менеджеры пакетов, файлы зависимостей и воспроизводимая сборка. Вы разберёте, почему проект работает на одной машине и падает на другой.</t>
         </is>
       </c>
       <c r="F47" s="5" t="inlineStr">
@@ -1455,7 +1455,7 @@
       </c>
       <c r="E48" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Студент проверяет чужой пул-реквест по чек-листу, оставляет замечания и собирает проект в релизную версию, сдаёт рецензию и артефакт сборки.</t>
+          <t xml:space="preserve">Вы проверяете чужой пул-реквест по чек-листу, оставляете замечания и собираете проект в релизную версию, сдаёте рецензию и артефакт сборки.</t>
         </is>
       </c>
       <c r="F48" s="5" t="inlineStr">
@@ -1485,7 +1485,7 @@
       </c>
       <c r="E49" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Настройки приложения отдельно от кода: файлы среды, переменные окружения и секреты. Студент научится запускать один код с разными параметрами.</t>
+          <t xml:space="preserve">Настройки приложения отдельно от кода: файлы среды, переменные окружения и секреты. Вы научитесь запускать один код с разными параметрами.</t>
         </is>
       </c>
       <c r="F49" s="5" t="inlineStr">
@@ -1515,7 +1515,7 @@
       </c>
       <c r="E50" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Путь приложения от репозитория до работающего сервера: сборка, артефакт, окружение и проверка после запуска. Студент разберёт, что ломается при переносе.</t>
+          <t xml:space="preserve">Путь приложения от репозитория до работающего сервера: сборка, артефакт, окружение и проверка после запуска. Вы разберёте, что ломается при переносе.</t>
         </is>
       </c>
       <c r="F50" s="5" t="inlineStr">
@@ -1545,7 +1545,7 @@
       </c>
       <c r="E51" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Студент готовит приложение к запуску: выносит настройки, собирает артефакт и запускает его на учебной машине, сдаёт инструкцию запуска и работающий сервис.</t>
+          <t xml:space="preserve">Вы готовите приложение к запуску: выносите настройки, собираете артефакт и запускаете его на учебной машине, сдаёте инструкцию запуска и работающий сервис.</t>
         </is>
       </c>
       <c r="F51" s="5" t="inlineStr">
@@ -1575,7 +1575,7 @@
       </c>
       <c r="E52" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Виды документации проекта: пользовательская, техническая и описание API. Студент научится выбирать адресата документа и писать инструкцию под его задачу.</t>
+          <t xml:space="preserve">Виды документации проекта: пользовательская, техническая и описание API. Вы научитесь выбирать адресата документа и писать инструкцию под его задачу.</t>
         </is>
       </c>
       <c r="F52" s="5" t="inlineStr">
@@ -1605,7 +1605,7 @@
       </c>
       <c r="E53" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Студент оформляет README с установкой и запуском, описывает API по шаблону и сдаёт документ, по которому другой человек поднимет проект с нуля.</t>
+          <t xml:space="preserve">Вы оформляете README с установкой и запуском, описываете API по шаблону и сдаёте документ, по которому другой человек поднимет проект с нуля.</t>
         </is>
       </c>
       <c r="F53" s="5" t="inlineStr">
@@ -1635,7 +1635,7 @@
       </c>
       <c r="E54" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Требования к итоговому проекту, состав модулей и критерии оценки. Студент составит план работ по проекту и распределит задачи по этапам.</t>
+          <t xml:space="preserve">Требования к итоговому проекту, состав модулей и критерии оценки. Вы составите план работ по проекту и распределите задачи по этапам.</t>
         </is>
       </c>
       <c r="F54" s="5" t="inlineStr">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="E55" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Студент выбирает тему индивидуального проекта, описывает назначение и пользователей системы, собирает каркас репозитория и сдаёт заявку с деревом каталогов.</t>
+          <t xml:space="preserve">Вы выбираете тему индивидуального проекта, описываете назначение и пользователей системы, собираете каркас репозитория и сдаёте заявку с деревом каталогов.</t>
         </is>
       </c>
       <c r="F55" s="5" t="inlineStr">
@@ -1695,7 +1695,7 @@
       </c>
       <c r="E56" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Студент проектирует схему базы проекта, создаёт таблицы и связи, добавляет модуль входа с хешированием пароля и сдаёт скрипт схемы и рабочий вход.</t>
+          <t xml:space="preserve">Вы проектируете схему базы проекта, создаёте таблицы и связи, добавляете модуль входа с хешированием пароля и сдаёте скрипт схемы и рабочий вход.</t>
         </is>
       </c>
       <c r="F56" s="5" t="inlineStr">
@@ -1725,7 +1725,7 @@
       </c>
       <c r="E57" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Студент реализует в проекте создание, чтение, изменение и удаление записей, добавляет проверку полей и сдаёт работающий модуль с набором проверенных сценариев.</t>
+          <t xml:space="preserve">Вы реализуете в проекте создание, чтение, изменение и удаление записей, добавляете проверку полей и сдаёте работающий модуль с набором проверенных сценариев.</t>
         </is>
       </c>
       <c r="F57" s="5" t="inlineStr">
@@ -1755,7 +1755,7 @@
       </c>
       <c r="E58" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Студент открывает функции проекта через API, добавляет единый формат ошибок и сдаёт коллекцию запросов, где видны успешные и ошибочные ответы.</t>
+          <t xml:space="preserve">Вы открываете функции проекта через API, добавляете единый формат ошибок и сдаёте коллекцию запросов, где видны успешные и ошибочные ответы.</t>
         </is>
       </c>
       <c r="F58" s="5" t="inlineStr">
@@ -1785,7 +1785,7 @@
       </c>
       <c r="E59" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Студент покрывает ключевые функции проекта тестами, добавляет в коллекцию Postman проверки ответа и сдаёт отчёт о прогоне тестов.</t>
+          <t xml:space="preserve">Вы покрываете ключевые функции проекта тестами, добавляете в коллекцию Postman проверки ответа и сдаёте отчёт о прогоне тестов.</t>
         </is>
       </c>
       <c r="F59" s="5" t="inlineStr">
@@ -1815,7 +1815,7 @@
       </c>
       <c r="E60" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Студент закрывает секреты проекта, включает проверку доступа и запускает приложение на учебной машине, сдаёт инструкцию запуска и отчёт о проверке безопасности.</t>
+          <t xml:space="preserve">Вы закрываете секреты проекта, включаете проверку доступа и запускаете приложение на учебной машине, сдаёте инструкцию запуска и отчёт о проверке безопасности.</t>
         </is>
       </c>
       <c r="F60" s="5" t="inlineStr">
@@ -1845,7 +1845,7 @@
       </c>
       <c r="E61" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Студент готовит документацию проекта и презентацию с демонстрацией работы, сдаёт README, описание API и слайды для защиты.</t>
+          <t xml:space="preserve">Вы готовите документацию проекта и презентацию с демонстрацией работы, сдаёте README, описание API и слайды для защиты.</t>
         </is>
       </c>
       <c r="F61" s="5" t="inlineStr">
@@ -1875,7 +1875,7 @@
       </c>
       <c r="E62" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Студент защищает индивидуальный проект: показывает работающее приложение, отвечает на вопросы по коду и архитектуре, сдаёт итоговый комплект документов.</t>
+          <t xml:space="preserve">Вы защищаете индивидуальный проект: показываете работающее приложение, отвечаете на вопросы по коду и архитектуре, сдаёте итоговый комплект документов.</t>
         </is>
       </c>
       <c r="F62" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Rework the МДК.05.02 plan before writing lessons
- rename practices so they no longer repeat lecture titles
- add an ORM practice after the ORM lecture
- shorten the environment practice to 90 minutes to keep 144 hours
- renumber chapters, directories and glyphs
</commit_message>
<xml_diff>
--- a/courses/3/is-code/dist/Учебный_план_Разработка_кода_информационных_систем.xlsx
+++ b/courses/3/is-code/dist/Учебный_план_Разработка_кода_информационных_систем.xlsx
@@ -109,7 +109,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:F63"/>
+  <dimension ref="A1:F64"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="7" customWidth="1"/>
@@ -307,7 +307,7 @@
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Практика 1. Структура проекта; Базовый Python</t>
+          <t xml:space="preserve">Практика 1. Каркас учебного проекта и первый модуль</t>
         </is>
       </c>
       <c r="D10" s="6">
@@ -357,7 +357,7 @@
     <row r="12" ht="60" customHeight="1">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">8-9</t>
+          <t xml:space="preserve">8</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
@@ -367,15 +367,15 @@
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Практика 2. Настройка VS Code; Настройка Visual Studio 2022</t>
+          <t xml:space="preserve">Практика 2. Рабочее окружение разработчика</t>
         </is>
       </c>
       <c r="D12" s="6">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Вы ставите расширения Python и C#, настраиваете интерпретатор, форматирование и отладчик в двух редакторах, сдаёте скриншоты настроек и запущенный проект.</t>
+          <t xml:space="preserve">Вы настраиваете два рабочих места: расширения Python в VS Code и проект C# в Visual Studio 2022, проверяете интерпретатор, форматирование и отладчик, сдаёте короткий протокол настроек и запущенный проект.</t>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr">
@@ -387,7 +387,7 @@
     <row r="13" ht="45" customHeight="1">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">10</t>
+          <t xml:space="preserve">9</t>
         </is>
       </c>
       <c r="B13" s="6" t="inlineStr">
@@ -417,7 +417,7 @@
     <row r="14" ht="45" customHeight="1">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">11</t>
+          <t xml:space="preserve">10</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
@@ -447,7 +447,7 @@
     <row r="15" ht="60" customHeight="1">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">12</t>
+          <t xml:space="preserve">11</t>
         </is>
       </c>
       <c r="B15" s="6" t="inlineStr">
@@ -477,7 +477,7 @@
     <row r="16" ht="60" customHeight="1">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">13-14</t>
+          <t xml:space="preserve">12-13</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr">
@@ -487,7 +487,7 @@
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Практика 3. Базовый C#; Функции</t>
+          <t xml:space="preserve">Практика 3. Консольный расчёт на C# с методами</t>
         </is>
       </c>
       <c r="D16" s="6">
@@ -507,7 +507,7 @@
     <row r="17" ht="45" customHeight="1">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">15</t>
+          <t xml:space="preserve">14</t>
         </is>
       </c>
       <c r="B17" s="6" t="inlineStr">
@@ -537,7 +537,7 @@
     <row r="18" ht="45" customHeight="1">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">16</t>
+          <t xml:space="preserve">15</t>
         </is>
       </c>
       <c r="B18" s="6" t="inlineStr">
@@ -547,7 +547,7 @@
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Практика 4. ООП</t>
+          <t xml:space="preserve">Практика 4. Модель предметной области в классах</t>
         </is>
       </c>
       <c r="D18" s="6">
@@ -567,7 +567,7 @@
     <row r="19" ht="45" customHeight="1">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">17</t>
+          <t xml:space="preserve">16</t>
         </is>
       </c>
       <c r="B19" s="6" t="inlineStr">
@@ -597,7 +597,7 @@
     <row r="20" ht="60" customHeight="1">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">18</t>
+          <t xml:space="preserve">17</t>
         </is>
       </c>
       <c r="B20" s="6" t="inlineStr">
@@ -607,7 +607,7 @@
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Практика 5. Исключения</t>
+          <t xml:space="preserve">Практика 5. Устойчивость программы к неверному вводу</t>
         </is>
       </c>
       <c r="D20" s="6">
@@ -627,7 +627,7 @@
     <row r="21" ht="45" customHeight="1">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">19</t>
+          <t xml:space="preserve">18</t>
         </is>
       </c>
       <c r="B21" s="6" t="inlineStr">
@@ -657,7 +657,7 @@
     <row r="22" ht="45" customHeight="1">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">20</t>
+          <t xml:space="preserve">19</t>
         </is>
       </c>
       <c r="B22" s="6" t="inlineStr">
@@ -667,7 +667,7 @@
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Практика 6. Файлы</t>
+          <t xml:space="preserve">Практика 6. Журнал операций в текстовом файле</t>
         </is>
       </c>
       <c r="D22" s="6">
@@ -687,7 +687,7 @@
     <row r="23" ht="45" customHeight="1">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">21</t>
+          <t xml:space="preserve">20</t>
         </is>
       </c>
       <c r="B23" s="6" t="inlineStr">
@@ -717,7 +717,7 @@
     <row r="24" ht="45" customHeight="1">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">22</t>
+          <t xml:space="preserve">21</t>
         </is>
       </c>
       <c r="B24" s="6" t="inlineStr">
@@ -727,7 +727,7 @@
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Практика 7. JSON/CSV</t>
+          <t xml:space="preserve">Практика 7. Обмен данными с внешней системой</t>
         </is>
       </c>
       <c r="D24" s="6">
@@ -747,7 +747,7 @@
     <row r="25" ht="45" customHeight="1">
       <c r="A25" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">23</t>
+          <t xml:space="preserve">22</t>
         </is>
       </c>
       <c r="B25" s="6" t="inlineStr">
@@ -777,7 +777,7 @@
     <row r="26" ht="45" customHeight="1">
       <c r="A26" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">24</t>
+          <t xml:space="preserve">23</t>
         </is>
       </c>
       <c r="B26" s="6" t="inlineStr">
@@ -787,7 +787,7 @@
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Практика 8. SQLite</t>
+          <t xml:space="preserve">Практика 8. Схема учебной базы и связи таблиц</t>
         </is>
       </c>
       <c r="D26" s="6">
@@ -807,7 +807,7 @@
     <row r="27" ht="45" customHeight="1">
       <c r="A27" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">25</t>
+          <t xml:space="preserve">24</t>
         </is>
       </c>
       <c r="B27" s="6" t="inlineStr">
@@ -837,7 +837,7 @@
     <row r="28" ht="45" customHeight="1">
       <c r="A28" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">26</t>
+          <t xml:space="preserve">25</t>
         </is>
       </c>
       <c r="B28" s="6" t="inlineStr">
@@ -847,7 +847,7 @@
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Практика 9. SQL-запросы из кода</t>
+          <t xml:space="preserve">Практика 9. Выборка и изменение данных из программы</t>
         </is>
       </c>
       <c r="D28" s="6">
@@ -867,47 +867,47 @@
     <row r="29" ht="45" customHeight="1">
       <c r="A29" s="6" t="inlineStr">
         <is>
+          <t xml:space="preserve">26</t>
+        </is>
+      </c>
+      <c r="B29" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Лекция</t>
+        </is>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Лекция 15. ORM</t>
+        </is>
+      </c>
+      <c r="D29" s="6">
+        <v>2</v>
+      </c>
+      <c r="E29" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Модель таблицы как класс, сессия и запросы вместо ручного SQL. Вы сравните ORM и чистый SQL и увидите, где какой подход уместен.</t>
+        </is>
+      </c>
+      <c r="F29" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">модель, сессия, миграция, связь, ленивая загрузка</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="60" customHeight="1">
+      <c r="A30" s="6" t="inlineStr">
+        <is>
           <t xml:space="preserve">27</t>
         </is>
       </c>
-      <c r="B29" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Лекция</t>
-        </is>
-      </c>
-      <c r="C29" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Лекция 15. ORM</t>
-        </is>
-      </c>
-      <c r="D29" s="6">
-        <v>2</v>
-      </c>
-      <c r="E29" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Модель таблицы как класс, сессия и запросы вместо ручного SQL. Вы сравните ORM и чистый SQL и увидите, где какой подход уместен.</t>
-        </is>
-      </c>
-      <c r="F29" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">модель, сессия, миграция, связь, ленивая загрузка</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="45" customHeight="1">
-      <c r="A30" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">28</t>
-        </is>
-      </c>
       <c r="B30" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Лекция</t>
+          <t xml:space="preserve">Практика</t>
         </is>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Лекция 16. HTTP и API</t>
+          <t xml:space="preserve">Практика 10. Модель таблицы и запросы через ORM</t>
         </is>
       </c>
       <c r="D30" s="6">
@@ -915,149 +915,149 @@
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Методы HTTP, заголовки, коды состояния и структура REST-ресурса. Вы проследите путь запроса от клиента до ответа и научитесь читать ответ API.</t>
+          <t xml:space="preserve">Вы описываете таблицу классом модели, выполняете выборку, добавление и изменение через сессию, сравниваете результат с эквивалентным SQL-запросом и сдаёте скрипт с обоими вариантами и таблицей сверки.</t>
         </is>
       </c>
       <c r="F30" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">метод, заголовок, код состояния, ресурс, REST</t>
+          <t xml:space="preserve">модель, сессия, выборка, сохранение, сравнение с SQL</t>
         </is>
       </c>
     </row>
     <row r="31" ht="45" customHeight="1">
       <c r="A31" s="6" t="inlineStr">
         <is>
+          <t xml:space="preserve">28</t>
+        </is>
+      </c>
+      <c r="B31" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Лекция</t>
+        </is>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Лекция 16. HTTP и API</t>
+        </is>
+      </c>
+      <c r="D31" s="6">
+        <v>2</v>
+      </c>
+      <c r="E31" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Методы HTTP, заголовки, коды состояния и структура REST-ресурса. Вы проследите путь запроса от клиента до ответа и научитесь читать ответ API.</t>
+        </is>
+      </c>
+      <c r="F31" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">метод, заголовок, код состояния, ресурс, REST</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="45" customHeight="1">
+      <c r="A32" s="6" t="inlineStr">
+        <is>
           <t xml:space="preserve">29</t>
         </is>
       </c>
-      <c r="B31" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Лекция</t>
-        </is>
-      </c>
-      <c r="C31" s="5" t="inlineStr">
+      <c r="B32" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Лекция</t>
+        </is>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Лекция 17. Flask/FastAPI</t>
         </is>
       </c>
-      <c r="D31" s="6">
-        <v>2</v>
-      </c>
-      <c r="E31" s="5" t="inlineStr">
+      <c r="D32" s="6">
+        <v>2</v>
+      </c>
+      <c r="E32" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Сравнение двух Python-фреймворков: маршруты, схемы данных и автоматическая документация. Вы выберете фреймворк под задачу и обоснуете выбор.</t>
         </is>
       </c>
-      <c r="F31" s="5" t="inlineStr">
+      <c r="F32" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">маршрут, схема данных, документация, валидация, асинхронность</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="60" customHeight="1">
-      <c r="A32" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">30-31</t>
-        </is>
-      </c>
-      <c r="B32" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Практика</t>
-        </is>
-      </c>
-      <c r="C32" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Практика 10. HTTP-клиент; Flask API</t>
-        </is>
-      </c>
-      <c r="D32" s="6">
-        <v>4</v>
-      </c>
-      <c r="E32" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Вы запускаете Flask-сервис с двумя маршрутами, обращаетесь к нему из HTTP-клиента и Postman и сдаёте коллекцию запросов с ответами и кодами состояния.</t>
-        </is>
-      </c>
-      <c r="F32" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">маршрут, GET, POST, код состояния, коллекция запросов</t>
         </is>
       </c>
     </row>
     <row r="33" ht="60" customHeight="1">
       <c r="A33" s="6" t="inlineStr">
         <is>
+          <t xml:space="preserve">30-31</t>
+        </is>
+      </c>
+      <c r="B33" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Практика</t>
+        </is>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Практика 11. Сервис на Flask и проверка запросов</t>
+        </is>
+      </c>
+      <c r="D33" s="6">
+        <v>4</v>
+      </c>
+      <c r="E33" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Вы запускаете Flask-сервис с двумя маршрутами, обращаетесь к нему из HTTP-клиента и Postman и сдаёте коллекцию запросов с ответами и кодами состояния.</t>
+        </is>
+      </c>
+      <c r="F33" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">маршрут, GET, POST, код состояния, коллекция запросов</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="60" customHeight="1">
+      <c r="A34" s="6" t="inlineStr">
+        <is>
           <t xml:space="preserve">32</t>
         </is>
       </c>
-      <c r="B33" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Лекция</t>
-        </is>
-      </c>
-      <c r="C33" s="5" t="inlineStr">
+      <c r="B34" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Лекция</t>
+        </is>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Лекция 18. ASP.NET Core</t>
         </is>
       </c>
-      <c r="D33" s="6">
-        <v>2</v>
-      </c>
-      <c r="E33" s="5" t="inlineStr">
+      <c r="D34" s="6">
+        <v>2</v>
+      </c>
+      <c r="E34" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Устройство приложения ASP.NET Core: конвейер обработки запроса, внедрение зависимостей и конфигурация. Вы разберёте, где подключить сервис и middleware.</t>
         </is>
       </c>
-      <c r="F33" s="5" t="inlineStr">
+      <c r="F34" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">middleware, конвейер, внедрение зависимостей, сервис, конфигурация</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="45" customHeight="1">
-      <c r="A34" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">33</t>
-        </is>
-      </c>
-      <c r="B34" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Практика</t>
-        </is>
-      </c>
-      <c r="C34" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Практика 11. ASP.NET API</t>
-        </is>
-      </c>
-      <c r="D34" s="6">
-        <v>2</v>
-      </c>
-      <c r="E34" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Вы создаёте контроллер ASP.NET с маршрутами чтения и записи, подключаете хранилище и сдаёте работающий сервис с проверкой запросов в Postman.</t>
-        </is>
-      </c>
-      <c r="F34" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">контроллер, действие, маршрутизация, код состояния, хранилище</t>
         </is>
       </c>
     </row>
     <row r="35" ht="45" customHeight="1">
       <c r="A35" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">34</t>
+          <t xml:space="preserve">33</t>
         </is>
       </c>
       <c r="B35" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Лекция</t>
+          <t xml:space="preserve">Практика</t>
         </is>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Лекция 19. Авторизация</t>
+          <t xml:space="preserve">Практика 12. Веб-сервис на C# с чтением и записью</t>
         </is>
       </c>
       <c r="D35" s="6">
@@ -1065,299 +1065,299 @@
       </c>
       <c r="E35" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Аутентификация и авторизация, хранение паролей и выдача токена. Вы разберёте поток входа и типичные ошибки при проверке прав доступа.</t>
+          <t xml:space="preserve">Вы создаёте контроллер ASP.NET с маршрутами чтения и записи, подключаете хранилище и сдаёте работающий сервис с проверкой запросов в Postman.</t>
         </is>
       </c>
       <c r="F35" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">аутентификация, хеш пароля, токен, права доступа, сессия</t>
+          <t xml:space="preserve">контроллер, действие, маршрутизация, код состояния, хранилище</t>
         </is>
       </c>
     </row>
     <row r="36" ht="45" customHeight="1">
       <c r="A36" s="6" t="inlineStr">
         <is>
+          <t xml:space="preserve">34</t>
+        </is>
+      </c>
+      <c r="B36" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Лекция</t>
+        </is>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Лекция 19. Авторизация</t>
+        </is>
+      </c>
+      <c r="D36" s="6">
+        <v>2</v>
+      </c>
+      <c r="E36" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Аутентификация и авторизация, хранение паролей и выдача токена. Вы разберёте поток входа и типичные ошибки при проверке прав доступа.</t>
+        </is>
+      </c>
+      <c r="F36" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">аутентификация, хеш пароля, токен, права доступа, сессия</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="45" customHeight="1">
+      <c r="A37" s="6" t="inlineStr">
+        <is>
           <t xml:space="preserve">35</t>
         </is>
       </c>
-      <c r="B36" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Лекция</t>
-        </is>
-      </c>
-      <c r="C36" s="5" t="inlineStr">
+      <c r="B37" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Лекция</t>
+        </is>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Лекция 20. Безопасность</t>
         </is>
       </c>
-      <c r="D36" s="6">
-        <v>2</v>
-      </c>
-      <c r="E36" s="5" t="inlineStr">
+      <c r="D37" s="6">
+        <v>2</v>
+      </c>
+      <c r="E37" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Основные угрозы веб-приложения: инъекции, утечка секретов и слабая проверка доступа. Вы научитесь находить уязвимость в коде и предлагать защиту.</t>
         </is>
       </c>
-      <c r="F36" s="5" t="inlineStr">
+      <c r="F37" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">инъекция, утечка секретов, права доступа, шифрование, защита</t>
-        </is>
-      </c>
-    </row>
-    <row r="37" ht="60" customHeight="1">
-      <c r="A37" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">36</t>
-        </is>
-      </c>
-      <c r="B37" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Лекция</t>
-        </is>
-      </c>
-      <c r="C37" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Лекция 21. Валидация</t>
-        </is>
-      </c>
-      <c r="D37" s="6">
-        <v>2</v>
-      </c>
-      <c r="E37" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Проверка данных на входе, в модели и в базе: обязательность, длина, диапазон и формат. Вы построите правило проверки и вернёте понятное сообщение об ошибке.</t>
-        </is>
-      </c>
-      <c r="F37" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">обязательность, формат, диапазон, сообщение об ошибке, схема</t>
         </is>
       </c>
     </row>
     <row r="38" ht="60" customHeight="1">
       <c r="A38" s="6" t="inlineStr">
         <is>
+          <t xml:space="preserve">36</t>
+        </is>
+      </c>
+      <c r="B38" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Лекция</t>
+        </is>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Лекция 21. Валидация</t>
+        </is>
+      </c>
+      <c r="D38" s="6">
+        <v>2</v>
+      </c>
+      <c r="E38" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Проверка данных на входе, в модели и в базе: обязательность, длина, диапазон и формат. Вы построите правило проверки и вернёте понятное сообщение об ошибке.</t>
+        </is>
+      </c>
+      <c r="F38" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">обязательность, формат, диапазон, сообщение об ошибке, схема</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="60" customHeight="1">
+      <c r="A39" s="6" t="inlineStr">
+        <is>
           <t xml:space="preserve">37-38</t>
         </is>
       </c>
-      <c r="B38" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Практика</t>
-        </is>
-      </c>
-      <c r="C38" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Практика 12. Авторизация; Валидация</t>
-        </is>
-      </c>
-      <c r="D38" s="6">
+      <c r="B39" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Практика</t>
+        </is>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Практика 13. Вход в систему и проверка полей</t>
+        </is>
+      </c>
+      <c r="D39" s="6">
         <v>4</v>
       </c>
-      <c r="E38" s="5" t="inlineStr">
+      <c r="E39" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Вы добавляете в API вход по логину и паролю, проверку токена и валидацию полей, сдаёте сервис, который отклоняет неверные данные с понятным кодом ошибки.</t>
         </is>
       </c>
-      <c r="F38" s="5" t="inlineStr">
+      <c r="F39" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">логин, пароль, токен, схема проверки, код ошибки</t>
         </is>
       </c>
     </row>
-    <row r="39" ht="45" customHeight="1">
-      <c r="A39" s="6" t="inlineStr">
+    <row r="40" ht="45" customHeight="1">
+      <c r="A40" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">39</t>
         </is>
       </c>
-      <c r="B39" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Лекция</t>
-        </is>
-      </c>
-      <c r="C39" s="5" t="inlineStr">
+      <c r="B40" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Лекция</t>
+        </is>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Лекция 22. Логирование</t>
         </is>
       </c>
-      <c r="D39" s="6">
-        <v>2</v>
-      </c>
-      <c r="E39" s="5" t="inlineStr">
+      <c r="D40" s="6">
+        <v>2</v>
+      </c>
+      <c r="E40" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Уровни сообщений, формат записи и место хранения журнала. Вы настроите логирование так, чтобы по записи можно было восстановить ход запроса.</t>
         </is>
       </c>
-      <c r="F39" s="5" t="inlineStr">
+      <c r="F40" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">уровень, формат записи, идентификатор запроса, журнал, ротация</t>
         </is>
       </c>
     </row>
-    <row r="40" ht="60" customHeight="1">
-      <c r="A40" s="6" t="inlineStr">
+    <row r="41" ht="60" customHeight="1">
+      <c r="A41" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">40-41</t>
         </is>
       </c>
-      <c r="B40" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Практика</t>
-        </is>
-      </c>
-      <c r="C40" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Практика 13. Безопасность; Логирование</t>
-        </is>
-      </c>
-      <c r="D40" s="6">
+      <c r="B41" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Практика</t>
+        </is>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Практика 14. Аудит доступа и защита секретов</t>
+        </is>
+      </c>
+      <c r="D41" s="6">
         <v>4</v>
       </c>
-      <c r="E40" s="5" t="inlineStr">
+      <c r="E41" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Вы закрываете уязвимые места сервиса: убираете секреты из кода, включаете проверку ввода и пишете события в журнал, сдаёте отчёт о проверке и файл лога.</t>
         </is>
       </c>
-      <c r="F40" s="5" t="inlineStr">
+      <c r="F41" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">секрет, инъекция, журнал, уровень события, аудит</t>
-        </is>
-      </c>
-    </row>
-    <row r="41" ht="45" customHeight="1">
-      <c r="A41" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">42</t>
-        </is>
-      </c>
-      <c r="B41" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Лекция</t>
-        </is>
-      </c>
-      <c r="C41" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Лекция 23. Тестирование кода</t>
-        </is>
-      </c>
-      <c r="D41" s="6">
-        <v>2</v>
-      </c>
-      <c r="E41" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Модульные и интеграционные тесты, покрытие и граничные значения. Вы научитесь отличать проверку одной функции от проверки связки модулей.</t>
-        </is>
-      </c>
-      <c r="F41" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">модульный тест, интеграционный тест, граничное значение, покрытие, утверждение</t>
         </is>
       </c>
     </row>
     <row r="42" ht="45" customHeight="1">
       <c r="A42" s="6" t="inlineStr">
         <is>
+          <t xml:space="preserve">42</t>
+        </is>
+      </c>
+      <c r="B42" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Лекция</t>
+        </is>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Лекция 23. Тестирование кода</t>
+        </is>
+      </c>
+      <c r="D42" s="6">
+        <v>2</v>
+      </c>
+      <c r="E42" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Модульные и интеграционные тесты, покрытие и граничные значения. Вы научитесь отличать проверку одной функции от проверки связки модулей.</t>
+        </is>
+      </c>
+      <c r="F42" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">модульный тест, интеграционный тест, граничное значение, покрытие, утверждение</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="45" customHeight="1">
+      <c r="A43" s="6" t="inlineStr">
+        <is>
           <t xml:space="preserve">43</t>
         </is>
       </c>
-      <c r="B42" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Лекция</t>
-        </is>
-      </c>
-      <c r="C42" s="5" t="inlineStr">
+      <c r="B43" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Лекция</t>
+        </is>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Лекция 24. Отладка</t>
         </is>
       </c>
-      <c r="D42" s="6">
-        <v>2</v>
-      </c>
-      <c r="E42" s="5" t="inlineStr">
+      <c r="D43" s="6">
+        <v>2</v>
+      </c>
+      <c r="E43" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Точки останова, пошаговое выполнение и просмотр стека вызовов в VS Code и Visual Studio. Вы найдёте причину дефекта без правок наугад.</t>
         </is>
       </c>
-      <c r="F42" s="5" t="inlineStr">
+      <c r="F43" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">точка останова, шаг с заходом, стек вызовов, значение переменной, дефект</t>
         </is>
       </c>
     </row>
-    <row r="43" ht="60" customHeight="1">
-      <c r="A43" s="6" t="inlineStr">
+    <row r="44" ht="60" customHeight="1">
+      <c r="A44" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">44-45</t>
         </is>
       </c>
-      <c r="B43" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Практика</t>
-        </is>
-      </c>
-      <c r="C43" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Практика 14. Тесты; Отладка</t>
-        </is>
-      </c>
-      <c r="D43" s="6">
+      <c r="B44" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Практика</t>
+        </is>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Практика 15. Проверка модулей и поиск дефекта</t>
+        </is>
+      </c>
+      <c r="D44" s="6">
         <v>4</v>
       </c>
-      <c r="E43" s="5" t="inlineStr">
+      <c r="E44" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Вы пишете тесты на функцию и на маршрут API, запускаете их и находите дефект по падающему тесту, сдаёте набор тестов и короткий отчёт о причине сбоя.</t>
         </is>
       </c>
-      <c r="F43" s="5" t="inlineStr">
+      <c r="F44" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">ожидаемый результат, проверка функции, прогон, отчёт, дефект</t>
-        </is>
-      </c>
-    </row>
-    <row r="44" ht="45" customHeight="1">
-      <c r="A44" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">46</t>
-        </is>
-      </c>
-      <c r="B44" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Лекция</t>
-        </is>
-      </c>
-      <c r="C44" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Лекция 25. Git и ветки</t>
-        </is>
-      </c>
-      <c r="D44" s="6">
-        <v>2</v>
-      </c>
-      <c r="E44" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ветки, слияние и разрешение конфликтов в общем репозитории. Вы разберёте схему ветвления и научитесь сводить изменения без потери чужой работы.</t>
-        </is>
-      </c>
-      <c r="F44" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ветка, слияние, конфликт, перебазирование, история коммитов</t>
         </is>
       </c>
     </row>
     <row r="45" ht="45" customHeight="1">
       <c r="A45" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">47</t>
+          <t xml:space="preserve">46</t>
         </is>
       </c>
       <c r="B45" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Практика</t>
+          <t xml:space="preserve">Лекция</t>
         </is>
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Практика 15. Git</t>
+          <t xml:space="preserve">Лекция 25. Git и ветки</t>
         </is>
       </c>
       <c r="D45" s="6">
@@ -1365,29 +1365,29 @@
       </c>
       <c r="E45" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Вы инициализируете репозиторий, делаете серию коммитов, отправляете проект на GitHub и сдаёте ссылку на репозиторий с историей изменений.</t>
+          <t xml:space="preserve">Ветки, слияние и разрешение конфликтов в общем репозитории. Вы разберёте схему ветвления и научитесь сводить изменения без потери чужой работы.</t>
         </is>
       </c>
       <c r="F45" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">репозиторий, коммит, индекс, удалённый репозиторий, gitignore</t>
+          <t xml:space="preserve">ветка, слияние, конфликт, перебазирование, история коммитов</t>
         </is>
       </c>
     </row>
     <row r="46" ht="45" customHeight="1">
       <c r="A46" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">48</t>
+          <t xml:space="preserve">47</t>
         </is>
       </c>
       <c r="B46" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Лекция</t>
+          <t xml:space="preserve">Практика</t>
         </is>
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Лекция 26. Code review</t>
+          <t xml:space="preserve">Практика 16. История изменений учебного проекта</t>
         </is>
       </c>
       <c r="D46" s="6">
@@ -1395,19 +1395,19 @@
       </c>
       <c r="E46" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Цели рецензирования, чек-лист и культура замечаний. Вы разберёте, чем полезное замечание отличается от придирки, и потренируетесь на фрагменте кода.</t>
+          <t xml:space="preserve">Вы инициализируете репозиторий, делаете серию коммитов, отправляете проект на GitHub и сдаёте ссылку на репозиторий с историей изменений.</t>
         </is>
       </c>
       <c r="F46" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">рецензия, чек-лист, дефект, стиль, обратная связь</t>
+          <t xml:space="preserve">репозиторий, коммит, индекс, удалённый репозиторий, gitignore</t>
         </is>
       </c>
     </row>
     <row r="47" ht="45" customHeight="1">
       <c r="A47" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">49</t>
+          <t xml:space="preserve">48</t>
         </is>
       </c>
       <c r="B47" s="6" t="inlineStr">
@@ -1417,7 +1417,7 @@
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Лекция 27. Сборка и зависимости</t>
+          <t xml:space="preserve">Лекция 26. Code review</t>
         </is>
       </c>
       <c r="D47" s="6">
@@ -1425,119 +1425,119 @@
       </c>
       <c r="E47" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Менеджеры пакетов, файлы зависимостей и воспроизводимая сборка. Вы разберёте, почему проект работает на одной машине и падает на другой.</t>
+          <t xml:space="preserve">Цели рецензирования, чек-лист и культура замечаний. Вы разберёте, чем полезное замечание отличается от придирки, и потренируетесь на фрагменте кода.</t>
         </is>
       </c>
       <c r="F47" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">пакет, версия, lock-файл, виртуальное окружение, воспроизводимость</t>
+          <t xml:space="preserve">рецензия, чек-лист, дефект, стиль, обратная связь</t>
         </is>
       </c>
     </row>
     <row r="48" ht="45" customHeight="1">
       <c r="A48" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">50-51</t>
+          <t xml:space="preserve">49</t>
         </is>
       </c>
       <c r="B48" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Практика</t>
+          <t xml:space="preserve">Лекция</t>
         </is>
       </c>
       <c r="C48" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Практика 16. Code review; Сборка</t>
+          <t xml:space="preserve">Лекция 27. Сборка и зависимости</t>
         </is>
       </c>
       <c r="D48" s="6">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E48" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Вы проверяете чужой пул-реквест по чек-листу, оставляете замечания и собираете проект в релизную версию, сдаёте рецензию и артефакт сборки.</t>
+          <t xml:space="preserve">Менеджеры пакетов, файлы зависимостей и воспроизводимая сборка. Вы разберёте, почему проект работает на одной машине и падает на другой.</t>
         </is>
       </c>
       <c r="F48" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">пул-реквест, чек-лист, замечание, релиз, артефакт</t>
+          <t xml:space="preserve">пакет, версия, lock-файл, виртуальное окружение, воспроизводимость</t>
         </is>
       </c>
     </row>
     <row r="49" ht="45" customHeight="1">
       <c r="A49" s="6" t="inlineStr">
         <is>
+          <t xml:space="preserve">50-51</t>
+        </is>
+      </c>
+      <c r="B49" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Практика</t>
+        </is>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Практика 17. Рецензия пул-реквеста и релизная сборка</t>
+        </is>
+      </c>
+      <c r="D49" s="6">
+        <v>4</v>
+      </c>
+      <c r="E49" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Вы проверяете чужой пул-реквест по чек-листу, оставляете замечания и собираете проект в релизную версию, сдаёте рецензию и артефакт сборки.</t>
+        </is>
+      </c>
+      <c r="F49" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">пул-реквест, чек-лист, замечание, релиз, артефакт</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="45" customHeight="1">
+      <c r="A50" s="6" t="inlineStr">
+        <is>
           <t xml:space="preserve">52</t>
         </is>
       </c>
-      <c r="B49" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Лекция</t>
-        </is>
-      </c>
-      <c r="C49" s="5" t="inlineStr">
+      <c r="B50" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Лекция</t>
+        </is>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Лекция 28. Конфигурация</t>
         </is>
       </c>
-      <c r="D49" s="6">
-        <v>2</v>
-      </c>
-      <c r="E49" s="5" t="inlineStr">
+      <c r="D50" s="6">
+        <v>2</v>
+      </c>
+      <c r="E50" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Настройки приложения отдельно от кода: файлы среды, переменные окружения и секреты. Вы научитесь запускать один код с разными параметрами.</t>
         </is>
       </c>
-      <c r="F49" s="5" t="inlineStr">
+      <c r="F50" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">файл настроек, переменная окружения, профиль, секрет, значение по умолчанию</t>
-        </is>
-      </c>
-    </row>
-    <row r="50" ht="60" customHeight="1">
-      <c r="A50" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">53</t>
-        </is>
-      </c>
-      <c r="B50" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Лекция</t>
-        </is>
-      </c>
-      <c r="C50" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Лекция 29. Развёртывание</t>
-        </is>
-      </c>
-      <c r="D50" s="6">
-        <v>2</v>
-      </c>
-      <c r="E50" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Путь приложения от репозитория до работающего сервера: сборка, артефакт, окружение и проверка после запуска. Вы разберёте, что ломается при переносе.</t>
-        </is>
-      </c>
-      <c r="F50" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">сборка, артефакт, окружение, порт, проверка запуска</t>
         </is>
       </c>
     </row>
     <row r="51" ht="60" customHeight="1">
       <c r="A51" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">54</t>
+          <t xml:space="preserve">53</t>
         </is>
       </c>
       <c r="B51" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Практика</t>
+          <t xml:space="preserve">Лекция</t>
         </is>
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Практика 17. Развёртывание</t>
+          <t xml:space="preserve">Лекция 29. Развёртывание</t>
         </is>
       </c>
       <c r="D51" s="6">
@@ -1545,141 +1545,141 @@
       </c>
       <c r="E51" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Вы готовите приложение к запуску: выносите настройки, собираете артефакт и запускаете его на учебной машине, сдаёте инструкцию запуска и работающий сервис.</t>
+          <t xml:space="preserve">Путь приложения от репозитория до работающего сервера: сборка, артефакт, окружение и проверка после запуска. Вы разберёте, что ломается при переносе.</t>
         </is>
       </c>
       <c r="F51" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">артефакт, настройки, порт, инструкция запуска, окружение</t>
+          <t xml:space="preserve">сборка, артефакт, окружение, порт, проверка запуска</t>
         </is>
       </c>
     </row>
     <row r="52" ht="60" customHeight="1">
       <c r="A52" s="6" t="inlineStr">
         <is>
+          <t xml:space="preserve">54</t>
+        </is>
+      </c>
+      <c r="B52" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Практика</t>
+        </is>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Практика 18. Запуск приложения на учебной машине</t>
+        </is>
+      </c>
+      <c r="D52" s="6">
+        <v>2</v>
+      </c>
+      <c r="E52" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Вы готовите приложение к запуску: выносите настройки, собираете артефакт и запускаете его на учебной машине, сдаёте инструкцию запуска и работающий сервис.</t>
+        </is>
+      </c>
+      <c r="F52" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">артефакт, настройки, порт, инструкция запуска, окружение</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="60" customHeight="1">
+      <c r="A53" s="6" t="inlineStr">
+        <is>
           <t xml:space="preserve">55</t>
         </is>
       </c>
-      <c r="B52" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Лекция</t>
-        </is>
-      </c>
-      <c r="C52" s="5" t="inlineStr">
+      <c r="B53" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Лекция</t>
+        </is>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Лекция 30. Документирование</t>
         </is>
       </c>
-      <c r="D52" s="6">
-        <v>2</v>
-      </c>
-      <c r="E52" s="5" t="inlineStr">
+      <c r="D53" s="6">
+        <v>2</v>
+      </c>
+      <c r="E53" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Виды документации проекта: пользовательская, техническая и описание API. Вы научитесь выбирать адресата документа и писать инструкцию под его задачу.</t>
         </is>
       </c>
-      <c r="F52" s="5" t="inlineStr">
+      <c r="F53" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">адресат, инструкция, описание API, руководство, полнота</t>
-        </is>
-      </c>
-    </row>
-    <row r="53" ht="45" customHeight="1">
-      <c r="A53" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">56</t>
-        </is>
-      </c>
-      <c r="B53" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Практика</t>
-        </is>
-      </c>
-      <c r="C53" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Практика 18. Документация</t>
-        </is>
-      </c>
-      <c r="D53" s="6">
-        <v>2</v>
-      </c>
-      <c r="E53" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Вы оформляете README с установкой и запуском, описываете API по шаблону и сдаёте документ, по которому другой человек поднимет проект с нуля.</t>
-        </is>
-      </c>
-      <c r="F53" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">README, установка, маршрут API, пример запроса, шаблон</t>
         </is>
       </c>
     </row>
     <row r="54" ht="45" customHeight="1">
       <c r="A54" s="6" t="inlineStr">
         <is>
+          <t xml:space="preserve">56</t>
+        </is>
+      </c>
+      <c r="B54" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Практика</t>
+        </is>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Практика 19. Инструкция запуска и описание API</t>
+        </is>
+      </c>
+      <c r="D54" s="6">
+        <v>2</v>
+      </c>
+      <c r="E54" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Вы оформляете README с установкой и запуском, описываете API по шаблону и сдаёте документ, по которому другой человек поднимет проект с нуля.</t>
+        </is>
+      </c>
+      <c r="F54" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">README, установка, маршрут API, пример запроса, шаблон</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="45" customHeight="1">
+      <c r="A55" s="6" t="inlineStr">
+        <is>
           <t xml:space="preserve">57</t>
         </is>
       </c>
-      <c r="B54" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Лекция</t>
-        </is>
-      </c>
-      <c r="C54" s="5" t="inlineStr">
+      <c r="B55" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Лекция</t>
+        </is>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Лекция 31. Итоговый проект</t>
         </is>
       </c>
-      <c r="D54" s="6">
-        <v>2</v>
-      </c>
-      <c r="E54" s="5" t="inlineStr">
+      <c r="D55" s="6">
+        <v>2</v>
+      </c>
+      <c r="E55" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Требования к итоговому проекту, состав модулей и критерии оценки. Вы составите план работ по проекту и распределите задачи по этапам.</t>
         </is>
       </c>
-      <c r="F54" s="5" t="inlineStr">
+      <c r="F55" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">требования, модуль, план работ, этап, критерии</t>
         </is>
       </c>
     </row>
-    <row r="55" ht="60" customHeight="1">
-      <c r="A55" s="6" t="inlineStr">
+    <row r="56" ht="60" customHeight="1">
+      <c r="A56" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">58-59</t>
         </is>
       </c>
-      <c r="B55" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Практика</t>
-        </is>
-      </c>
-      <c r="C55" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Практика 19. Индивидуальный проект: выбор темы; структура проекта</t>
-        </is>
-      </c>
-      <c r="D55" s="6">
-        <v>4</v>
-      </c>
-      <c r="E55" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Вы выбираете тему индивидуального проекта, описываете назначение и пользователей системы, собираете каркас репозитория и сдаёте заявку с деревом каталогов.</t>
-        </is>
-      </c>
-      <c r="F55" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">тема проекта, пользователь, границы системы, каркас, заявка</t>
-        </is>
-      </c>
-    </row>
-    <row r="56" ht="45" customHeight="1">
-      <c r="A56" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">60-61</t>
-        </is>
-      </c>
       <c r="B56" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">Практика</t>
@@ -1687,7 +1687,7 @@
       </c>
       <c r="C56" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Практика 20. Индивидуальный проект: база данных; модуль авторизации</t>
+          <t xml:space="preserve">Практика 20. Заявка и каркас индивидуального проекта</t>
         </is>
       </c>
       <c r="D56" s="6">
@@ -1695,19 +1695,19 @@
       </c>
       <c r="E56" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Вы проектируете схему базы проекта, создаёте таблицы и связи, добавляете модуль входа с хешированием пароля и сдаёте скрипт схемы и рабочий вход.</t>
+          <t xml:space="preserve">Вы выбираете тему индивидуального проекта, описываете назначение и пользователей системы, собираете каркас репозитория и сдаёте заявку с деревом каталогов.</t>
         </is>
       </c>
       <c r="F56" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">схема, ключ, справочник, хеш, вход</t>
-        </is>
-      </c>
-    </row>
-    <row r="57" ht="60" customHeight="1">
+          <t xml:space="preserve">тема проекта, пользователь, границы системы, каркас, заявка</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="45" customHeight="1">
       <c r="A57" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">62-63</t>
+          <t xml:space="preserve">60-61</t>
         </is>
       </c>
       <c r="B57" s="6" t="inlineStr">
@@ -1717,7 +1717,7 @@
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Практика 21. Индивидуальный проект: CRUD; валидация</t>
+          <t xml:space="preserve">Практика 21. Схема базы и вход в индивидуальном проекте</t>
         </is>
       </c>
       <c r="D57" s="6">
@@ -1725,19 +1725,19 @@
       </c>
       <c r="E57" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Вы реализуете в проекте создание, чтение, изменение и удаление записей, добавляете проверку полей и сдаёте работающий модуль с набором проверенных сценариев.</t>
+          <t xml:space="preserve">Вы проектируете схему базы проекта, создаёте таблицы и связи, добавляете модуль входа с хешированием пароля и сдаёте скрипт схемы и рабочий вход.</t>
         </is>
       </c>
       <c r="F57" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">создание, чтение, изменение, удаление, проверка поля</t>
-        </is>
-      </c>
-    </row>
-    <row r="58" ht="45" customHeight="1">
+          <t xml:space="preserve">схема, ключ, справочник, хеш, вход</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="60" customHeight="1">
       <c r="A58" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">64-65</t>
+          <t xml:space="preserve">62-63</t>
         </is>
       </c>
       <c r="B58" s="6" t="inlineStr">
@@ -1747,7 +1747,7 @@
       </c>
       <c r="C58" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Практика 22. Индивидуальный проект: API; обработка ошибок</t>
+          <t xml:space="preserve">Практика 22. Операции CRUD и проверка полей в проекте</t>
         </is>
       </c>
       <c r="D58" s="6">
@@ -1755,19 +1755,19 @@
       </c>
       <c r="E58" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Вы открываете функции проекта через API, добавляете единый формат ошибок и сдаёте коллекцию запросов, где видны успешные и ошибочные ответы.</t>
+          <t xml:space="preserve">Вы реализуете в проекте создание, чтение, изменение и удаление записей, добавляете проверку полей и сдаёте работающий модуль с набором проверенных сценариев.</t>
         </is>
       </c>
       <c r="F58" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">маршрут, формат ошибки, код состояния, сценарий, коллекция</t>
+          <t xml:space="preserve">создание, чтение, изменение, удаление, проверка поля</t>
         </is>
       </c>
     </row>
     <row r="59" ht="45" customHeight="1">
       <c r="A59" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">66-67</t>
+          <t xml:space="preserve">64-65</t>
         </is>
       </c>
       <c r="B59" s="6" t="inlineStr">
@@ -1777,7 +1777,7 @@
       </c>
       <c r="C59" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Практика 23. Индивидуальный проект: тесты; Postman</t>
+          <t xml:space="preserve">Практика 23. API проекта и единый формат ошибок</t>
         </is>
       </c>
       <c r="D59" s="6">
@@ -1785,19 +1785,19 @@
       </c>
       <c r="E59" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Вы покрываете ключевые функции проекта тестами, добавляете в коллекцию Postman проверки ответа и сдаёте отчёт о прогоне тестов.</t>
+          <t xml:space="preserve">Вы открываете функции проекта через API, добавляете единый формат ошибок и сдаёте коллекцию запросов, где видны успешные и ошибочные ответы.</t>
         </is>
       </c>
       <c r="F59" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">проверка функции, проверка ответа, коллекция, прогон, отчёт</t>
-        </is>
-      </c>
-    </row>
-    <row r="60" ht="60" customHeight="1">
+          <t xml:space="preserve">маршрут, формат ошибки, код состояния, сценарий, коллекция</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="45" customHeight="1">
       <c r="A60" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">68-69</t>
+          <t xml:space="preserve">66-67</t>
         </is>
       </c>
       <c r="B60" s="6" t="inlineStr">
@@ -1807,7 +1807,7 @@
       </c>
       <c r="C60" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Практика 24. Индивидуальный проект: безопасность; развёртывание</t>
+          <t xml:space="preserve">Практика 24. Тесты и коллекция Postman для проекта</t>
         </is>
       </c>
       <c r="D60" s="6">
@@ -1815,19 +1815,19 @@
       </c>
       <c r="E60" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Вы закрываете секреты проекта, включаете проверку доступа и запускаете приложение на учебной машине, сдаёте инструкцию запуска и отчёт о проверке безопасности.</t>
+          <t xml:space="preserve">Вы покрываете ключевые функции проекта тестами, добавляете в коллекцию Postman проверки ответа и сдаёте отчёт о прогоне тестов.</t>
         </is>
       </c>
       <c r="F60" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">секрет, роль, доступ, инструкция, запуск</t>
-        </is>
-      </c>
-    </row>
-    <row r="61" ht="45" customHeight="1">
+          <t xml:space="preserve">проверка функции, проверка ответа, коллекция, прогон, отчёт</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="60" customHeight="1">
       <c r="A61" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">70-71</t>
+          <t xml:space="preserve">68-69</t>
         </is>
       </c>
       <c r="B61" s="6" t="inlineStr">
@@ -1837,7 +1837,7 @@
       </c>
       <c r="C61" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Практика 25. Индивидуальный проект: документация; презентация</t>
+          <t xml:space="preserve">Практика 25. Защита доступа и запуск проекта</t>
         </is>
       </c>
       <c r="D61" s="6">
@@ -1845,82 +1845,112 @@
       </c>
       <c r="E61" s="5" t="inlineStr">
         <is>
+          <t xml:space="preserve">Вы закрываете секреты проекта, включаете проверку доступа и запускаете приложение на учебной машине, сдаёте инструкцию запуска и отчёт о проверке безопасности.</t>
+        </is>
+      </c>
+      <c r="F61" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">секрет, роль, доступ, инструкция, запуск</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="45" customHeight="1">
+      <c r="A62" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">70-71</t>
+        </is>
+      </c>
+      <c r="B62" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Практика</t>
+        </is>
+      </c>
+      <c r="C62" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Практика 26. Документация и презентация проекта</t>
+        </is>
+      </c>
+      <c r="D62" s="6">
+        <v>4</v>
+      </c>
+      <c r="E62" s="5" t="inlineStr">
+        <is>
           <t xml:space="preserve">Вы готовите документацию проекта и презентацию с демонстрацией работы, сдаёте README, описание API и слайды для защиты.</t>
         </is>
       </c>
-      <c r="F61" s="5" t="inlineStr">
+      <c r="F62" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">README, описание API, слайд, демонстрация, структура доклада</t>
         </is>
       </c>
     </row>
-    <row r="62" ht="60" customHeight="1">
-      <c r="A62" s="6" t="inlineStr">
+    <row r="63" ht="60" customHeight="1">
+      <c r="A63" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">72</t>
         </is>
       </c>
-      <c r="B62" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Практика</t>
-        </is>
-      </c>
-      <c r="C62" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Практика 26. Индивидуальный проект: защита</t>
-        </is>
-      </c>
-      <c r="D62" s="6">
-        <v>2</v>
-      </c>
-      <c r="E62" s="5" t="inlineStr">
+      <c r="B63" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Практика</t>
+        </is>
+      </c>
+      <c r="C63" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Практика 27. Защита индивидуального проекта</t>
+        </is>
+      </c>
+      <c r="D63" s="6">
+        <v>2</v>
+      </c>
+      <c r="E63" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Вы защищаете индивидуальный проект: показываете работающее приложение, отвечаете на вопросы по коду и архитектуре, сдаёте итоговый комплект документов.</t>
         </is>
       </c>
-      <c r="F62" s="5" t="inlineStr">
+      <c r="F63" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">демонстрация, сценарий, архитектура, вопросы, комплект документов</t>
         </is>
       </c>
     </row>
-    <row r="63" ht="22" customHeight="1">
-      <c r="A63" s="7" t="inlineStr">
+    <row r="64" ht="22" customHeight="1">
+      <c r="A64" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Итого</t>
         </is>
       </c>
-      <c r="B63" s="7" t="inlineStr">
+      <c r="B64" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="C63" s="7" t="inlineStr">
+      <c r="C64" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="D63" s="6">
+      <c r="D64" s="6">
         <v>144</v>
       </c>
-      <c r="E63" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">57 позиций</t>
-        </is>
-      </c>
-      <c r="F63" s="5" t="inlineStr">
+      <c r="E64" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">58 позиций</t>
+        </is>
+      </c>
+      <c r="F64" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A5:F62"/>
+  <autoFilter ref="A5:F63"/>
   <mergeCells count="4">
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A3:F3"/>
-    <mergeCell ref="A63:C63"/>
+    <mergeCell ref="A64:C64"/>
   </mergeCells>
   <pageMargins left="0.5" right="0.5" top="0.6" bottom="0.6" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>